<commit_message>
TASK-Clean up and Fix everything
Cleaned up all the models and data.
Fixed everything for future updates.
</commit_message>
<xml_diff>
--- a/20-excel-based/models/060-authorization-model.xlsx
+++ b/20-excel-based/models/060-authorization-model.xlsx
@@ -14331,7 +14331,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
-  <dimension ref="B2:L52"/>
+  <dimension ref="B2:L53"/>
   <sheetFormatPr defaultRowHeight="21.75" customHeight="1"/>
   <cols>
     <col min="1" max="1" customWidth="true" width="10.08203125"/>
@@ -15606,12 +15606,12 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>emrspllineitem</t>
+          <t>emspiritem</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>emattrspir</t>
+          <t>emattrbusinessimpact</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
@@ -15653,7 +15653,7 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>emattrpr</t>
+          <t>emattrspir</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
@@ -15695,7 +15695,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>emattrno</t>
+          <t>emattrpr</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
@@ -15737,7 +15737,7 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>emattrrspl</t>
+          <t>emattrno</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
@@ -15747,7 +15747,7 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
@@ -15779,7 +15779,7 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>emattrtemplinkup</t>
+          <t>emattrrspl</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
@@ -15789,7 +15789,7 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
@@ -15821,7 +15821,7 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>emattrtempsystemupdateddate</t>
+          <t>emattrtemplinkup</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -15861,14 +15861,9 @@
           <t>emrspllineitem</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>emrelbelongstopritem</t>
-        </is>
-      </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t/>
+          <t>emattrtempsystemupdateddate</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -15878,12 +15873,12 @@
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
@@ -15905,12 +15900,17 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>emplantitem</t>
+          <t>emrspllineitem</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>emrelbelongstopritem</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>emattrspir</t>
+          <t/>
         </is>
       </c>
       <c r="H37" t="inlineStr">
@@ -15920,12 +15920,12 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
@@ -15952,7 +15952,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>emattrpr</t>
+          <t>emattrspir</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -15994,7 +15994,7 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>emattrno</t>
+          <t>emattrpr</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
@@ -16036,7 +16036,7 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>emattrrspl</t>
+          <t>emattrno</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
@@ -16078,7 +16078,7 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>emattrtemplinkup</t>
+          <t>emattrrspl</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
@@ -16120,7 +16120,7 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>emattrtempsystemupdateddate</t>
+          <t>emattrtemplinkup</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
@@ -16157,12 +16157,12 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>emrefsupplier</t>
+          <t>emplantitem</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>refattrhassubproject</t>
+          <t>emattrtempsystemupdateddate</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
@@ -16177,7 +16177,7 @@
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
@@ -16199,12 +16199,12 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>emspir</t>
+          <t>emrefsupplier</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>emattrspir</t>
+          <t>refattrhassubproject</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
@@ -16219,7 +16219,7 @@
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
@@ -16246,7 +16246,7 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>emattrpr</t>
+          <t>emattrspir</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
@@ -16288,7 +16288,7 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>emattrno</t>
+          <t>emattrpr</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
@@ -16330,7 +16330,7 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>emattrrspl</t>
+          <t>emattrno</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
@@ -16372,7 +16372,7 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>emattrtemplinkup</t>
+          <t>emattrrspl</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
@@ -16414,7 +16414,7 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>emattrtempsystemupdateddate</t>
+          <t>emattrtemplinkup</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
@@ -16456,12 +16456,12 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>emattrisapprovedforspir</t>
+          <t>emattrtempsystemupdateddate</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
@@ -16481,7 +16481,7 @@
       </c>
       <c r="L50" t="inlineStr">
         <is>
-          <t/>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -16493,27 +16493,27 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>emprtsupplier</t>
+          <t>emspir</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>prtattrreacentsubproject</t>
+          <t>emattrisapprovedforspir</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="K51" t="inlineStr">
@@ -16523,7 +16523,7 @@
       </c>
       <c r="L51" t="inlineStr">
         <is>
-          <t>No</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -16540,30 +16540,72 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
+          <t>prtattrreacentsubproject</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>systemadmin</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>emprtsupplier</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
           <t>prtattrallothersubproject</t>
         </is>
       </c>
-      <c r="H52" t="inlineStr">
+      <c r="H53" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="I52" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="J52" t="inlineStr">
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="K52" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="L52" t="inlineStr">
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L53" t="inlineStr">
         <is>
           <t>No</t>
         </is>

</xml_diff>